<commit_message>
Update Upload Transaction Data template
</commit_message>
<xml_diff>
--- a/capital-gains/Upload Data.xlsx
+++ b/capital-gains/Upload Data.xlsx
@@ -1,26 +1,59 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AnkitKulshrestha\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD351507-76A6-4944-BF07-B2450426E1C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B52283A-C29C-4C6D-BE99-0E8A365D0241}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="23054" yWindow="0" windowWidth="30715" windowHeight="18842" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25974" yWindow="-109" windowWidth="26301" windowHeight="14169" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={6445E355-957D-417D-91EF-92F47C5161F1}</author>
+  </authors>
+  <commentList>
+    <comment ref="H3" authorId="0" shapeId="0" xr:uid="{6445E355-957D-417D-91EF-92F47C5161F1}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    RBA Rates
+Reply:
+    https://www.rba.gov.au/statistics/historical-data.html</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="14">
   <si>
     <t>Side</t>
   </si>
@@ -37,9 +70,6 @@
     <t>Fee Currency</t>
   </si>
   <si>
-    <t>BTC-USD</t>
-  </si>
-  <si>
     <t>Buy</t>
   </si>
   <si>
@@ -56,13 +86,25 @@
   </si>
   <si>
     <t>Exchange Rates</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QQQ </t>
+  </si>
+  <si>
+    <t xml:space="preserve">NDQ </t>
+  </si>
+  <si>
+    <t>AUD</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+  </numFmts>
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -74,6 +116,24 @@
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -93,16 +153,23 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="3">
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="2" xr:uid="{8E36A078-107E-417B-8067-EFC7273DC6CF}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -115,6 +182,12 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Ankit Kulshrestha" id="{60629866-0BB1-4839-8031-ABE6AD240EA3}" userId="S::ankit@acebiz.com.au::aee89e21-9e45-49dd-85ec-dfc3e48f973b" providerId="AD"/>
+</personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -313,12 +386,29 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="H3" dT="2025-10-28T22:09:59.75" personId="{60629866-0BB1-4839-8031-ABE6AD240EA3}" id="{6445E355-957D-417D-91EF-92F47C5161F1}">
+    <text>RBA Rates</text>
+  </threadedComment>
+  <threadedComment ref="H3" dT="2025-10-28T22:10:01.39" personId="{60629866-0BB1-4839-8031-ABE6AD240EA3}" id="{ACD3E018-254A-41D9-B4E4-A966F2E8B7F2}" parentId="{6445E355-957D-417D-91EF-92F47C5161F1}">
+    <text>https://www.rba.gov.au/statistics/historical-data.html</text>
+    <extLst>
+      <x:ext xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" uri="{F7C98A9C-CBB3-438F-8F68-D28B6AF4A901}">
+        <xltc2:checksum>2799957553</xltc2:checksum>
+        <xltc2:hyperlink startIndex="0" length="54" url="https://www.rba.gov.au/statistics/historical-data.html"/>
+      </x:ext>
+    </extLst>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr defaultColWidth="12.625" defaultRowHeight="15.8" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.75" customWidth="1"/>
@@ -327,10 +417,10 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>9</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>10</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
@@ -348,56 +438,132 @@
         <v>4</v>
       </c>
       <c r="H1" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="12.9" x14ac:dyDescent="0.2">
+      <c r="A2" s="2">
+        <v>45524</v>
+      </c>
+      <c r="B2" t="s">
         <v>11</v>
       </c>
+      <c r="C2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="4">
+        <v>1</v>
+      </c>
+      <c r="E2" s="1">
+        <v>900</v>
+      </c>
+      <c r="F2" s="1">
+        <v>3</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>6</v>
+      </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" s="2">
+    <row r="3" spans="1:8" ht="15.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2">
+        <v>45519</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" s="5">
+        <v>2</v>
+      </c>
+      <c r="E3">
+        <v>938.14</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H3" s="3">
+        <v>1.5129999999999999</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="15.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
+        <v>45519</v>
+      </c>
+      <c r="B4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="5">
+        <v>2</v>
+      </c>
+      <c r="E4">
+        <v>938.14</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H4" s="3">
+        <v>1.5129999999999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="15.8" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="2">
         <v>45516</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="1">
-        <v>1</v>
-      </c>
-      <c r="E2" s="1">
-        <v>1000</v>
-      </c>
-      <c r="F2" s="1">
-        <v>5</v>
-      </c>
-      <c r="G2" s="1" t="s">
+      <c r="D5" s="5">
+        <v>39</v>
+      </c>
+      <c r="E5">
+        <v>1631.76</v>
+      </c>
+      <c r="F5" s="1">
+        <v>3</v>
+      </c>
+      <c r="G5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="15.8" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="2">
+        <v>45638</v>
+      </c>
+      <c r="B6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" s="2">
-        <v>45610</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" s="1">
-        <v>1</v>
-      </c>
-      <c r="E3" s="1">
-        <v>900</v>
-      </c>
-      <c r="F3" s="1">
+      <c r="D6" s="5">
+        <v>39</v>
+      </c>
+      <c r="E6">
+        <v>1631.76</v>
+      </c>
+      <c r="F6" s="1">
         <v>3</v>
       </c>
-      <c r="G3" s="1" t="s">
-        <v>7</v>
+      <c r="G6" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>